<commit_message>
added spearman's rho cross compution for cost and environmental since they are closely correlated then updated paper graphs and made it a lot clearer in many areas. also removed redundant areas, made clarity edits,
</commit_message>
<xml_diff>
--- a/Output Files DeepSeek V4 Flash/metrics_summary_deepseek.xlsx
+++ b/Output Files DeepSeek V4 Flash/metrics_summary_deepseek.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D246"/>
+  <dimension ref="A1:D270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4421,7 +4421,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Example-Guided_LLM_Scoring</t>
+          <t>Direct_LLM_Scoring</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -4431,17 +4431,17 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>match_content</t>
+          <t>cross_criterion_rho_overall</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>195</v>
+        <v>0.9202</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Example-Guided_LLM_Scoring</t>
+          <t>Direct_LLM_Scoring</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>match_no_match</t>
+          <t>cross_criterion_rho_pvalue</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -4461,7 +4461,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Example-Guided_LLM_Scoring</t>
+          <t>Direct_LLM_Scoring</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -4471,17 +4471,17 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>diag_files_loaded</t>
+          <t>cross_criterion_rho_HVAC</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>5</v>
+        <v>0.9992</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Example-Guided_LLM_Scoring</t>
+          <t>Direct_LLM_Scoring</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -4491,17 +4491,17 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>diag_total_scenarios</t>
+          <t>cross_criterion_rho_HVAC_pvalue</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>975</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Example-Guided_LLM_Scoring</t>
+          <t>Direct_LLM_Scoring</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -4511,17 +4511,17 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>diag_failed_scenarios</t>
+          <t>cross_criterion_rho_Appliance</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>0</v>
+        <v>0.8988</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Example-Guided_LLM_Scoring</t>
+          <t>Direct_LLM_Scoring</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -4531,17 +4531,17 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>diag_successful_scenarios</t>
+          <t>cross_criterion_rho_Appliance_pvalue</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>975</v>
+        <v>0</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Example-Guided_LLM_Scoring</t>
+          <t>Direct_LLM_Scoring</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -4551,17 +4551,17 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>diag_failed_calls</t>
+          <t>cross_criterion_rho_Shower</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>0</v>
+        <v>0.9661999999999999</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Example-Guided_LLM_Scoring</t>
+          <t>Direct_LLM_Scoring</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -4571,11 +4571,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>diag_successful_calls</t>
+          <t>cross_criterion_rho_Shower_pvalue</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>2925</v>
+        <v>0</v>
       </c>
     </row>
     <row r="209">
@@ -4591,11 +4591,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>diag_EXTRACTION_INVALID_JSON</t>
+          <t>match_content</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>0</v>
+        <v>195</v>
       </c>
     </row>
     <row r="210">
@@ -4611,7 +4611,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>diag_FAILED_MISSING_SCORE</t>
+          <t>match_no_match</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -4631,11 +4631,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>diag_FAILED_OUT_OF_BOUNDS</t>
+          <t>diag_files_loaded</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="212">
@@ -4651,11 +4651,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>diag_FAILED_INVALID_SCORE_TYPE</t>
+          <t>diag_total_scenarios</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>0</v>
+        <v>975</v>
       </c>
     </row>
     <row r="213">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>diag_FAILED_API_EXHAUSTED</t>
+          <t>diag_failed_scenarios</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -4691,11 +4691,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>diag_FAILED_UNKNOWN</t>
+          <t>diag_successful_scenarios</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>0</v>
+        <v>975</v>
       </c>
     </row>
     <row r="215">
@@ -4711,11 +4711,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>n_runs</t>
+          <t>diag_failed_calls</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="216">
@@ -4731,11 +4731,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>n_successful_runs_mean</t>
+          <t>diag_successful_calls</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>5</v>
+        <v>2925</v>
       </c>
     </row>
     <row r="217">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>n_failed_scenarios</t>
+          <t>diag_EXTRACTION_INVALID_JSON</t>
         </is>
       </c>
       <c r="D217" t="n">
@@ -4771,11 +4771,11 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>n_total_arch_scenarios</t>
+          <t>diag_FAILED_MISSING_SCORE</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>195</v>
+        <v>0</v>
       </c>
     </row>
     <row r="219">
@@ -4791,7 +4791,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>total_failure_rate</t>
+          <t>diag_FAILED_OUT_OF_BOUNDS</t>
         </is>
       </c>
       <c r="D219" t="n">
@@ -4801,7 +4801,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -4811,17 +4811,17 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>match_content</t>
+          <t>diag_FAILED_INVALID_SCORE_TYPE</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>195</v>
+        <v>0</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>match_no_match</t>
+          <t>diag_FAILED_API_EXHAUSTED</t>
         </is>
       </c>
       <c r="D221" t="n">
@@ -4841,7 +4841,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -4851,17 +4851,17 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>diag_files_loaded</t>
+          <t>diag_FAILED_UNKNOWN</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -4871,17 +4871,17 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>diag_total_scenarios</t>
+          <t>n_runs</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>975</v>
+        <v>5</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -4891,17 +4891,17 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>diag_failed_scenarios</t>
+          <t>n_successful_runs_mean</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -4911,17 +4911,17 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>diag_successful_scenarios</t>
+          <t>n_failed_scenarios</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>974</v>
+        <v>0</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -4931,17 +4931,17 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>diag_failed_calls</t>
+          <t>n_total_arch_scenarios</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>1</v>
+        <v>195</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -4951,17 +4951,17 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>diag_successful_calls</t>
+          <t>total_failure_rate</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>974</v>
+        <v>0</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -4971,17 +4971,17 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>diag_FAILED_EXTRACTION_NON_JSON_WRAPPER</t>
+          <t>cross_criterion_rho_overall</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>0</v>
+        <v>0.9202</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -4991,7 +4991,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>diag_EXTRACTION_INVALID_JSON</t>
+          <t>cross_criterion_rho_pvalue</t>
         </is>
       </c>
       <c r="D229" t="n">
@@ -5001,7 +5001,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -5011,17 +5011,17 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>diag_FAILED_EXTRACTION_INVALID_DECISION_TYPE</t>
+          <t>cross_criterion_rho_HVAC</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>0</v>
+        <v>0.9992</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -5031,7 +5031,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>diag_FAILED_EXTRACTION_INVALID_CALCULATOR</t>
+          <t>cross_criterion_rho_HVAC_pvalue</t>
         </is>
       </c>
       <c r="D231" t="n">
@@ -5041,7 +5041,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -5051,17 +5051,17 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>diag_FAILED_EXTRACTION_MISSING_PARAMETERS</t>
+          <t>cross_criterion_rho_Appliance</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>0</v>
+        <v>0.8988</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -5071,7 +5071,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>diag_FAILED_EXTRACTION_EXCEPTION</t>
+          <t>cross_criterion_rho_Appliance_pvalue</t>
         </is>
       </c>
       <c r="D233" t="n">
@@ -5081,7 +5081,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -5091,17 +5091,17 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>diag_FAILED_GROUND_TRUTH_CALCULATION_EXCEPTION</t>
+          <t>cross_criterion_rho_Shower</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>0</v>
+        <v>0.9661999999999999</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>LLM-Parameterized_Reference_Scoring</t>
+          <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>diag_FAILED_GROUND_TRUTH_MISSING_KEY</t>
+          <t>cross_criterion_rho_Shower_pvalue</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -5131,11 +5131,11 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>diag_FAILED_API_EXHAUSTED</t>
+          <t>match_content</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>0</v>
+        <v>195</v>
       </c>
     </row>
     <row r="237">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>diag_FAILED_UNKNOWN</t>
+          <t>match_no_match</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>n_runs</t>
+          <t>diag_files_loaded</t>
         </is>
       </c>
       <c r="D238" t="n">
@@ -5191,11 +5191,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>n_successful_runs_mean</t>
+          <t>diag_total_scenarios</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>4.99</v>
+        <v>975</v>
       </c>
     </row>
     <row r="240">
@@ -5211,11 +5211,11 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>n_failed_scenarios</t>
+          <t>diag_failed_scenarios</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="241">
@@ -5231,11 +5231,11 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>n_total_arch_scenarios</t>
+          <t>diag_successful_scenarios</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>195</v>
+        <v>974</v>
       </c>
     </row>
     <row r="242">
@@ -5251,11 +5251,11 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>total_failure_rate</t>
+          <t>diag_failed_calls</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="243">
@@ -5271,11 +5271,11 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>extraction_failure_rate</t>
+          <t>diag_successful_calls</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>0</v>
+        <v>974</v>
       </c>
     </row>
     <row r="244">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>calculation_failure_rate</t>
+          <t>diag_FAILED_EXTRACTION_NON_JSON_WRAPPER</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>n_extraction_failures</t>
+          <t>diag_EXTRACTION_INVALID_JSON</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -5331,10 +5331,490 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
+          <t>diag_FAILED_EXTRACTION_INVALID_DECISION_TYPE</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>diag_FAILED_EXTRACTION_INVALID_CALCULATOR</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>diag_FAILED_EXTRACTION_MISSING_PARAMETERS</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>diag_FAILED_EXTRACTION_EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>diag_FAILED_GROUND_TRUTH_CALCULATION_EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>diag_FAILED_GROUND_TRUTH_MISSING_KEY</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>diag_FAILED_API_EXHAUSTED</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>diag_FAILED_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>n_runs</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>n_successful_runs_mean</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>4.99</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>n_failed_scenarios</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>n_total_arch_scenarios</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>total_failure_rate</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>extraction_failure_rate</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>calculation_failure_rate</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>n_extraction_failures</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
           <t>n_calculation_failures</t>
         </is>
       </c>
-      <c r="D246" t="n">
+      <c r="D262" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>cross_criterion_rho_overall</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>0.9202</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>cross_criterion_rho_pvalue</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>cross_criterion_rho_HVAC</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>0.9992</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>cross_criterion_rho_HVAC_pvalue</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>cross_criterion_rho_Appliance</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>0.8988</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>cross_criterion_rho_Appliance_pvalue</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>cross_criterion_rho_Shower</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>0.9661999999999999</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>cross_criterion_rho_Shower_pvalue</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>